<commit_message>
highlighted things I will order in green on bom, yellow for sample
</commit_message>
<xml_diff>
--- a/01-main_board/main_board_v4/DigikeyOrdering/BOM-main_board_v3.xlsx
+++ b/01-main_board/main_board_v4/DigikeyOrdering/BOM-main_board_v3.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emma/Documents/JHU/22xt_kicad/01-main_board/main_board_v3/DigikeyOrdering/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\teais\22xt_kicad\01-main_board\main_board_v4\DigikeyOrdering\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{34C7EF8D-1F13-8045-BD7D-DE6C37C5C6E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDA21836-CC01-449E-84A3-02FD4744E13A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="35840" windowHeight="22400" xr2:uid="{E864DD15-E767-464B-8250-0CE0FF16D1D0}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{E864DD15-E767-464B-8250-0CE0FF16D1D0}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM-main_board_v3" sheetId="1" r:id="rId1"/>
@@ -744,7 +744,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -927,6 +927,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1091,10 +1103,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1471,12 +1484,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B7D0AEF-84B1-A34B-99F2-910B57565FEC}">
   <dimension ref="A1:I109"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="8" max="8" width="14.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1502,7 +1515,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>71</v>
       </c>
@@ -1519,7 +1532,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -1536,7 +1549,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>31</v>
       </c>
@@ -1553,7 +1566,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>19</v>
       </c>
@@ -1570,7 +1583,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>43</v>
       </c>
@@ -1585,7 +1598,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>26</v>
       </c>
@@ -1602,7 +1615,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>43</v>
       </c>
@@ -1617,7 +1630,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>43</v>
       </c>
@@ -1632,7 +1645,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>43</v>
       </c>
@@ -1647,7 +1660,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>43</v>
       </c>
@@ -1662,7 +1675,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>43</v>
       </c>
@@ -1677,7 +1690,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>43</v>
       </c>
@@ -1692,7 +1705,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>43</v>
       </c>
@@ -1707,7 +1720,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>43</v>
       </c>
@@ -1722,7 +1735,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>43</v>
       </c>
@@ -1737,7 +1750,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>43</v>
       </c>
@@ -1752,7 +1765,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>43</v>
       </c>
@@ -1767,7 +1780,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>43</v>
       </c>
@@ -1782,7 +1795,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>43</v>
       </c>
@@ -1797,7 +1810,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>43</v>
       </c>
@@ -1812,7 +1825,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>43</v>
       </c>
@@ -1827,7 +1840,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>43</v>
       </c>
@@ -1842,7 +1855,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>43</v>
       </c>
@@ -1857,7 +1870,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>43</v>
       </c>
@@ -1872,7 +1885,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>43</v>
       </c>
@@ -1887,7 +1900,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>43</v>
       </c>
@@ -1902,7 +1915,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>43</v>
       </c>
@@ -1917,28 +1930,27 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A29" s="2" t="s">
+    <row r="29" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="B29" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C29" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2">
-        <v>1</v>
-      </c>
-      <c r="G29">
+      <c r="C29" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E29" s="3">
+        <v>1</v>
+      </c>
+      <c r="G29" s="3">
         <v>10</v>
       </c>
-      <c r="H29" t="s">
+      <c r="H29" s="3" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>43</v>
       </c>
@@ -1953,7 +1965,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>43</v>
       </c>
@@ -1968,7 +1980,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>43</v>
       </c>
@@ -1983,7 +1995,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>43</v>
       </c>
@@ -1998,7 +2010,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>43</v>
       </c>
@@ -2013,7 +2025,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>43</v>
       </c>
@@ -2028,7 +2040,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>43</v>
       </c>
@@ -2043,7 +2055,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>43</v>
       </c>
@@ -2058,7 +2070,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>145</v>
       </c>
@@ -2075,7 +2087,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>145</v>
       </c>
@@ -2092,7 +2104,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>67</v>
       </c>
@@ -2109,7 +2121,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
         <v>43</v>
       </c>
@@ -2124,7 +2136,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
         <v>43</v>
       </c>
@@ -2139,41 +2151,41 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
+    <row r="43" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B43" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="C43" t="s">
+      <c r="C43" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="E43">
-        <v>1</v>
-      </c>
-      <c r="G43">
+      <c r="E43" s="3">
+        <v>1</v>
+      </c>
+      <c r="G43" s="3">
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
+    <row r="44" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B44" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="C44" t="s">
+      <c r="C44" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="E44">
-        <v>1</v>
-      </c>
-      <c r="G44">
+      <c r="E44" s="3">
+        <v>1</v>
+      </c>
+      <c r="G44" s="3">
         <v>3</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>117</v>
       </c>
@@ -2190,27 +2202,30 @@
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
+    <row r="46" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B46" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C46" t="s">
+      <c r="C46" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E46">
-        <v>1</v>
-      </c>
-      <c r="G46">
-        <v>1</v>
-      </c>
-      <c r="I46" t="s">
+      <c r="E46" s="2">
+        <v>1</v>
+      </c>
+      <c r="G46" s="2">
+        <v>1</v>
+      </c>
+      <c r="H46" s="2">
+        <v>2</v>
+      </c>
+      <c r="I46" s="2" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>133</v>
       </c>
@@ -2230,7 +2245,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>56</v>
       </c>
@@ -2247,27 +2262,27 @@
         <v>7</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
+    <row r="49" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B49" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C49" t="s">
+      <c r="C49" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="D49" t="s">
+      <c r="D49" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E49">
-        <v>1</v>
-      </c>
-      <c r="G49">
+      <c r="E49" s="3">
+        <v>1</v>
+      </c>
+      <c r="G49" s="3">
         <v>3</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>56</v>
       </c>
@@ -2284,7 +2299,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>47</v>
       </c>
@@ -2304,58 +2319,58 @@
         <v>3</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
+    <row r="52" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="B52" t="s">
+      <c r="B52" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="C52" t="s">
+      <c r="C52" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="E52">
-        <v>1</v>
-      </c>
-      <c r="G52">
+      <c r="E52" s="3">
+        <v>1</v>
+      </c>
+      <c r="G52" s="3">
         <v>3</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
+    <row r="53" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B53" t="s">
+      <c r="B53" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="C53" t="s">
+      <c r="C53" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="E53">
-        <v>1</v>
-      </c>
-      <c r="G53">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A54" t="s">
+      <c r="E53" s="3">
+        <v>1</v>
+      </c>
+      <c r="G53" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="B54" t="s">
+      <c r="B54" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C54" t="s">
+      <c r="C54" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="E54">
-        <v>1</v>
-      </c>
-      <c r="G54">
+      <c r="E54" s="3">
+        <v>1</v>
+      </c>
+      <c r="G54" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>99</v>
       </c>
@@ -2375,7 +2390,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>89</v>
       </c>
@@ -2392,24 +2407,24 @@
         <v>17</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A57" t="s">
+    <row r="57" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B57" t="s">
+      <c r="B57" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C57" t="s">
-        <v>11</v>
-      </c>
-      <c r="D57" t="s">
+      <c r="C57" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D57" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E57">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E57" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>69</v>
       </c>
@@ -2426,38 +2441,38 @@
         <v>191</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A59" t="s">
+    <row r="59" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B59" t="s">
+      <c r="B59" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C59" t="s">
-        <v>11</v>
-      </c>
-      <c r="D59" t="s">
+      <c r="C59" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D59" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E59">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A60">
+      <c r="E59" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="1">
         <v>47</v>
       </c>
-      <c r="B60" t="s">
+      <c r="B60" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="C60" t="s">
-        <v>11</v>
-      </c>
-      <c r="E60">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="C60" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E60" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>110</v>
       </c>
@@ -2471,7 +2486,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>110</v>
       </c>
@@ -2485,7 +2500,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>110</v>
       </c>
@@ -2499,7 +2514,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>110</v>
       </c>
@@ -2513,7 +2528,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>110</v>
       </c>
@@ -2527,21 +2542,21 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A66">
+    <row r="66" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="1">
         <v>47</v>
       </c>
-      <c r="B66" t="s">
+      <c r="B66" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="C66" t="s">
+      <c r="C66" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="E66">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E66" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>51</v>
       </c>
@@ -2558,7 +2573,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>51</v>
       </c>
@@ -2575,7 +2590,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>51</v>
       </c>
@@ -2592,7 +2607,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>51</v>
       </c>
@@ -2609,21 +2624,24 @@
         <v>50</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A71" t="s">
+    <row r="71" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B71" t="s">
+      <c r="B71" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C71" t="s">
-        <v>11</v>
-      </c>
-      <c r="E71">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="C71" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E71" s="3">
+        <v>1</v>
+      </c>
+      <c r="H71" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>110</v>
       </c>
@@ -2637,41 +2655,41 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A73" t="s">
+    <row r="73" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A73" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="B73" t="s">
+      <c r="B73" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C73" t="s">
-        <v>11</v>
-      </c>
-      <c r="E73">
-        <v>1</v>
-      </c>
-      <c r="G73">
+      <c r="C73" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E73" s="1">
+        <v>1</v>
+      </c>
+      <c r="G73" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A74" t="s">
+    <row r="74" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A74" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="B74" t="s">
+      <c r="B74" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="C74" t="s">
-        <v>11</v>
-      </c>
-      <c r="E74">
-        <v>1</v>
-      </c>
-      <c r="G74">
+      <c r="C74" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E74" s="1">
+        <v>1</v>
+      </c>
+      <c r="G74" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>110</v>
       </c>
@@ -2685,7 +2703,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>115</v>
       </c>
@@ -2702,7 +2720,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>110</v>
       </c>
@@ -2716,7 +2734,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>110</v>
       </c>
@@ -2730,7 +2748,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>110</v>
       </c>
@@ -2744,21 +2762,21 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A80" t="s">
+    <row r="80" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A80" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B80" t="s">
+      <c r="B80" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="C80" t="s">
-        <v>11</v>
-      </c>
-      <c r="E80">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="C80" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E80" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>110</v>
       </c>
@@ -2772,7 +2790,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>51</v>
       </c>
@@ -2785,8 +2803,11 @@
       <c r="E82">
         <v>1</v>
       </c>
-    </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G82">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>51</v>
       </c>
@@ -2799,8 +2820,11 @@
       <c r="E83">
         <v>1</v>
       </c>
-    </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G83">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>110</v>
       </c>
@@ -2814,191 +2838,191 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A85" t="s">
+    <row r="85" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A85" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B85" t="s">
+      <c r="B85" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C85" t="s">
-        <v>11</v>
-      </c>
-      <c r="D85" t="s">
+      <c r="C85" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D85" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="E85">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A86" t="s">
+      <c r="E85" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A86" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="B86" t="s">
+      <c r="B86" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="C86" t="s">
-        <v>11</v>
-      </c>
-      <c r="E86">
-        <v>1</v>
-      </c>
-      <c r="G86">
+      <c r="C86" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E86" s="1">
+        <v>1</v>
+      </c>
+      <c r="G86" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A87" t="s">
+    <row r="87" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A87" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="B87" t="s">
+      <c r="B87" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="C87" t="s">
-        <v>11</v>
-      </c>
-      <c r="E87">
-        <v>1</v>
-      </c>
-      <c r="G87">
+      <c r="C87" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E87" s="1">
+        <v>1</v>
+      </c>
+      <c r="G87" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A88" t="s">
+    <row r="88" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A88" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="B88" t="s">
+      <c r="B88" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="C88" t="s">
-        <v>11</v>
-      </c>
-      <c r="E88">
-        <v>1</v>
-      </c>
-      <c r="G88">
+      <c r="C88" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E88" s="1">
+        <v>1</v>
+      </c>
+      <c r="G88" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A89" t="s">
+    <row r="89" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A89" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="B89" t="s">
+      <c r="B89" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="C89" t="s">
-        <v>11</v>
-      </c>
-      <c r="E89">
-        <v>1</v>
-      </c>
-      <c r="G89">
+      <c r="C89" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E89" s="1">
+        <v>1</v>
+      </c>
+      <c r="G89" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A90" t="s">
+    <row r="90" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A90" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="B90" t="s">
+      <c r="B90" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="C90" t="s">
-        <v>11</v>
-      </c>
-      <c r="E90">
-        <v>1</v>
-      </c>
-      <c r="G90">
+      <c r="C90" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E90" s="1">
+        <v>1</v>
+      </c>
+      <c r="G90" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A91" t="s">
+    <row r="91" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A91" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="B91" t="s">
+      <c r="B91" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="C91" t="s">
-        <v>11</v>
-      </c>
-      <c r="E91">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A92" t="s">
+      <c r="C91" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E91" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A92" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="B92" t="s">
+      <c r="B92" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="C92" t="s">
-        <v>11</v>
-      </c>
-      <c r="E92">
-        <v>1</v>
-      </c>
-      <c r="G92">
+      <c r="C92" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E92" s="1">
+        <v>1</v>
+      </c>
+      <c r="G92" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A93" t="s">
+    <row r="93" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A93" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="B93" t="s">
+      <c r="B93" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="C93" t="s">
-        <v>11</v>
-      </c>
-      <c r="E93">
-        <v>1</v>
-      </c>
-      <c r="G93">
+      <c r="C93" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E93" s="1">
+        <v>1</v>
+      </c>
+      <c r="G93" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A94" t="s">
+    <row r="94" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A94" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="B94" t="s">
+      <c r="B94" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="C94" t="s">
-        <v>11</v>
-      </c>
-      <c r="E94">
-        <v>1</v>
-      </c>
-      <c r="G94">
+      <c r="C94" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E94" s="1">
+        <v>1</v>
+      </c>
+      <c r="G94" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A95">
+    <row r="95" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A95" s="1">
         <v>120</v>
       </c>
-      <c r="B95" t="s">
+      <c r="B95" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C95" t="s">
+      <c r="C95" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D95" t="s">
+      <c r="D95" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="E95">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E95" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>159</v>
       </c>
@@ -3015,109 +3039,115 @@
         <v>25</v>
       </c>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A97" t="s">
+    <row r="97" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A97" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B97" t="s">
+      <c r="B97" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C97" t="s">
-        <v>11</v>
-      </c>
-      <c r="D97" t="s">
+      <c r="C97" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D97" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E97">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A98" t="s">
+      <c r="E97" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A98" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="B98" t="s">
+      <c r="B98" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="C98" t="s">
-        <v>11</v>
-      </c>
-      <c r="E98">
-        <v>1</v>
-      </c>
-      <c r="G98">
+      <c r="C98" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E98" s="1">
+        <v>1</v>
+      </c>
+      <c r="G98" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A99" t="s">
+    <row r="99" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A99" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="B99" t="s">
+      <c r="B99" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="C99" t="s">
-        <v>11</v>
-      </c>
-      <c r="E99">
-        <v>1</v>
-      </c>
-      <c r="G99">
+      <c r="C99" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E99" s="1">
+        <v>1</v>
+      </c>
+      <c r="G99" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A100" t="s">
+    <row r="100" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A100" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="B100" t="s">
+      <c r="B100" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C100" t="s">
-        <v>11</v>
-      </c>
-      <c r="E100">
-        <v>1</v>
-      </c>
-      <c r="G100">
+      <c r="C100" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E100" s="1">
+        <v>1</v>
+      </c>
+      <c r="G100" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A101" t="s">
+    <row r="101" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A101" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="B101" t="s">
+      <c r="B101" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="C101" t="s">
-        <v>11</v>
-      </c>
-      <c r="E101">
-        <v>1</v>
-      </c>
-      <c r="G101">
+      <c r="C101" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E101" s="3">
+        <v>1</v>
+      </c>
+      <c r="G101" s="3">
         <v>25</v>
       </c>
-    </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A102" t="s">
+      <c r="H101" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A102" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="B102" t="s">
+      <c r="B102" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="C102" t="s">
-        <v>11</v>
-      </c>
-      <c r="E102">
-        <v>1</v>
-      </c>
-      <c r="G102">
+      <c r="C102" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E102" s="3">
+        <v>1</v>
+      </c>
+      <c r="G102" s="3">
         <v>10</v>
       </c>
-    </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H102" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="103" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>62</v>
       </c>
@@ -3131,24 +3161,24 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A104">
+    <row r="104" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A104" s="3">
         <v>749013011</v>
       </c>
-      <c r="B104" t="s">
+      <c r="B104" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C104">
+      <c r="C104" s="3">
         <v>749013011</v>
       </c>
-      <c r="E104">
-        <v>1</v>
-      </c>
-      <c r="G104">
+      <c r="E104" s="3">
+        <v>1</v>
+      </c>
+      <c r="G104" s="3">
         <v>3</v>
       </c>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>105</v>
       </c>
@@ -3168,24 +3198,27 @@
         <v>2</v>
       </c>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A106" t="s">
+    <row r="106" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A106" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="B106" t="s">
+      <c r="B106" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="C106" t="s">
+      <c r="C106" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="E106">
-        <v>1</v>
-      </c>
-      <c r="G106">
+      <c r="E106" s="2">
+        <v>1</v>
+      </c>
+      <c r="G106" s="2">
         <v>3</v>
       </c>
-    </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H106" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>122</v>
       </c>
@@ -3202,40 +3235,40 @@
         <v>192</v>
       </c>
     </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A108" t="s">
+    <row r="108" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A108" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B108" t="s">
+      <c r="B108" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="C108" t="s">
+      <c r="C108" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="E108">
-        <v>1</v>
-      </c>
-      <c r="G108">
+      <c r="E108" s="3">
+        <v>1</v>
+      </c>
+      <c r="G108" s="3">
         <v>4</v>
       </c>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A109" t="s">
+    <row r="109" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A109" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="B109" t="s">
+      <c r="B109" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="C109" t="s">
+      <c r="C109" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="E109">
-        <v>1</v>
-      </c>
-      <c r="G109">
-        <v>1</v>
-      </c>
-      <c r="H109" t="s">
+      <c r="E109" s="3">
+        <v>1</v>
+      </c>
+      <c r="G109" s="3">
+        <v>2</v>
+      </c>
+      <c r="H109" s="3" t="s">
         <v>193</v>
       </c>
     </row>

</xml_diff>